<commit_message>
Add 8 unidentified share.google grant links as a Triage group; commit generator
Adds the eight share.google links Lara supplied as placeholder rows in a new
"Triage" group (Workstream = Triage): link preserved, Status = Researching,
Next Action = resolve+verify, with funder/amount/deadline/fit left blank because
the redirects are blocked by this session's egress policy and could not be
resolved. A Summary line counts the triage group. The artifact now renders an
"Unidentified links — to resolve" section (58 rows total).

Also commits scripts/generate_dashboard.py (previously only in scratchpad and
lost on session reset) so the read-only HTML view can be regenerated from the
workbook in future sessions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uh1jFHPZFJnmJ5vxj2WzQC
</commit_message>
<xml_diff>
--- a/Funding_Dashboard.xlsx
+++ b/Funding_Dashboard.xlsx
@@ -156,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -188,6 +188,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -570,6 +574,46 @@
       <text>
         <t>~$5K-$50K per group; members join larger rounds.
 Search-verified via official-domain content (www.broadway-angels.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.broadway-angels.com/</t>
+      </text>
+    </comment>
+    <comment ref="J52" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/9zSHYE5KA0gu5XX5V</t>
+      </text>
+    </comment>
+    <comment ref="J53" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/s7xWCT7crmTazEj7t</t>
+      </text>
+    </comment>
+    <comment ref="J54" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/AM8yfJTwPWBEThxfl</t>
+      </text>
+    </comment>
+    <comment ref="J55" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/1mw6JD6kJkYIlH9TR</t>
+      </text>
+    </comment>
+    <comment ref="J56" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/CerWenXESJ13cRnhZ</t>
+      </text>
+    </comment>
+    <comment ref="J57" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/SQdBs8RhlxauVQNqX</t>
+      </text>
+    </comment>
+    <comment ref="J58" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/6WnqpweYBP2E7sbhw</t>
+      </text>
+    </comment>
+    <comment ref="J59" authorId="0" shapeId="0">
+      <text>
+        <t>Link could not be opened in this session: share.google redirect blocked by egress policy on 2026-09-22. Paste the destination URL or the grant name so it can be verified and scored. Source (unresolved): https://share.google/xRA7UAMRJAnQkyusM</t>
       </text>
     </comment>
   </commentList>
@@ -944,6 +988,22 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Unidentified grant links (share.google) - to resolve &amp; categorize</t>
+        </is>
+      </c>
+      <c r="C18" s="15">
+        <f>COUNTIF('Funding Dashboard'!A2:A500,"Triage")</f>
+        <v/>
+      </c>
+    </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -977,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -4562,6 +4622,390 @@
       <c r="O51" t="inlineStr">
         <is>
           <t>https://www.broadway-angels.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Grant to identify #1 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J52" t="n"/>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Resolve link #1 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>https://share.google/9zSHYE5KA0gu5XX5V</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Grant to identify #2 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J53" t="n"/>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Resolve link #2 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>https://share.google/s7xWCT7crmTazEj7t</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Grant to identify #3 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J54" t="n"/>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Resolve link #3 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>https://share.google/AM8yfJTwPWBEThxfl</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Grant to identify #4 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J55" t="n"/>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Resolve link #4 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>https://share.google/1mw6JD6kJkYIlH9TR</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Grant to identify #5 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J56" t="n"/>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Resolve link #5 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>https://share.google/CerWenXESJ13cRnhZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Grant to identify #6 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J57" t="n"/>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Resolve link #6 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>https://share.google/SQdBs8RhlxauVQNqX</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Grant to identify #7 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J58" t="n"/>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Resolve link #7 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>https://share.google/6WnqpweYBP2E7sbhw</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Triage</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Grant to identify #8 (share.google link)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Unknown - resolve link</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Grant (unverified)</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Unidentified - the share.google redirect could not be opened in this session (egress policy). Resolve the URL to determine funder, entity/incorporation/ownership/visa eligibility, amount, and deadline before this row is treated as fact.</t>
+        </is>
+      </c>
+      <c r="J59" t="n"/>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Resolve link #8 (open it or paste the destination URL / grant name); then verify funder, amount, deadline, and eligibility.</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>https://share.google/xRA7UAMRJAnQkyusM</t>
         </is>
       </c>
     </row>

</xml_diff>